<commit_message>
Remove module docstring and update spreadsheet
</commit_message>
<xml_diff>
--- a/empleados.xlsx
+++ b/empleados.xlsx
@@ -480,7 +480,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Soldador</t>
+          <t>Administrativo</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -490,10 +490,10 @@
         <v>46096</v>
       </c>
       <c r="G2" t="n">
-        <v>90000</v>
+        <v>50000</v>
       </c>
       <c r="H2" t="n">
-        <v>2700000</v>
+        <v>1500000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>